<commit_message>
Premium and marketing only: gift weights, quarter results, market news
- Decisions are now the premium (base + 19 coefficients) and the campaign:
  marketing budget, media share and a weight for each gift. Channel focus,
  claims operations, reinsurance, NPS and capital are gone; two trophies.
- The decision workbook drops the Claim sheet; old workbooks are refused.
- Quarter reviews keep the quarter's results table on stage, with team
  status and brochures in a strip; teams upload brochures from their page.
- The live feed becomes market news (events only); detailed results show
  one category at a time; the app type is IBM Plex Sans.
- Audit workbook, AI rivals, balance test, samples and participant data
  follow the new model.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/samples/casco-decision-sample.xlsx
+++ b/dist/samples/casco-decision-sample.xlsx
@@ -8,14 +8,10 @@
     <sheet name="Input" sheetId="1" r:id="rId1"/>
     <sheet name="Premium" sheetId="2" r:id="rId2"/>
     <sheet name="Marketing" sheetId="3" r:id="rId3"/>
-    <sheet name="Claim" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="CoefficientList">Premium!$XFD$1:$XFD$41</definedName>
-    <definedName name="FocusList">Marketing!$XFC$1:$XFC$19</definedName>
-    <definedName name="OfferList">Marketing!$XFD$1:$XFD$4</definedName>
     <definedName name="PercentageList">Marketing!$XFB$1:$XFB$21</definedName>
-    <definedName name="YesNoList">Claim!$XFD$1:$XFD$2</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -155,7 +151,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -318,40 +314,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF004894"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF004894"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF004894"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF004894"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -444,7 +411,7 @@
     <xf numFmtId="9" fontId="8" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -460,63 +427,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -600,27 +510,11 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Set the marketing budget and its channel distribution (each channel min 10%, total must = 100%), and the digital campaign</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24.8" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3️⃣</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CLAIM</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Set the claims operations budget and choose the quota-share reinsurance</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">Set the marketing budget, split it among media &amp; offer (total must = 100%) and weight the gifts (total must = 100%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24.8" customHeight="1"/>
     <row r="11" ht="30" customHeight="1">
       <c r="B11" s="7" t="inlineStr">
         <is>
@@ -648,7 +542,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marketing channels total must equal 100%; media + offer must equal 100%.</t>
+          <t xml:space="preserve">Media + offer must equal 100%; the gift weights must equal 100%.</t>
         </is>
       </c>
     </row>
@@ -660,7 +554,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marketing + claims operations + reinsurance fee must stay within the decision budget (€1,022,000).</t>
+          <t xml:space="preserve">The marketing budget must stay within €1,022,000.</t>
         </is>
       </c>
     </row>
@@ -703,7 +597,7 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Follow the market’s price structure, grow through agents.</t>
+          <t xml:space="preserve">Follow the market’s price structure, grow through the campaign.</t>
         </is>
       </c>
     </row>
@@ -1227,7 +1121,7 @@
     <col min="7" max="7" width="31.9" customWidth="1"/>
     <col min="9" max="9" width="10.3" customWidth="1"/>
     <col min="10" max="10" width="8.1" customWidth="1"/>
-    <col min="11" max="11" width="16.1" customWidth="1"/>
+    <col min="11" max="11" width="12.6" customWidth="1"/>
     <col min="12" max="12" width="11.3" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1235,64 +1129,32 @@
       <c r="XFB1" s="23">
         <v>0</v>
       </c>
-      <c r="XFC1" s="23">
-        <v>0.1</v>
-      </c>
-      <c r="XFD1" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Discount on concert/event</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="35.2" customHeight="1">
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARKETING - CHANNEL DISTRIBUTION</t>
+          <t xml:space="preserve">MARKETING - MEDIA &amp; OFFER</t>
         </is>
       </c>
       <c r="XFB2" s="23">
         <v>0.05</v>
       </c>
-      <c r="XFC2" s="23">
-        <v>0.15</v>
-      </c>
-      <c r="XFD2" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Restaurant gift card</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="37.2" customHeight="1">
       <c r="B3" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Your marketing budget buys visibility in the sales channels and can run a digital campaign.
-Split the campaign among media &amp; offer. Sum should equal to 100%.</t>
+          <t xml:space="preserve">You have a budget of up to €1,022,000. You will split this among media &amp; offer.
+Sum should equal to 100%. Then weight the gifts: their sum should also equal to 100%.</t>
         </is>
       </c>
       <c r="XFB3" s="23">
         <v>0.1</v>
-      </c>
-      <c r="XFC3" s="23">
-        <v>0.2</v>
-      </c>
-      <c r="XFD3" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Coffee gift card</t>
-        </is>
       </c>
     </row>
     <row r="4">
       <c r="XFB4" s="23">
         <v>0.15</v>
       </c>
-      <c r="XFC4" s="23">
-        <v>0.25</v>
-      </c>
-      <c r="XFD4" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Discount on gym membership</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="42.6" customHeight="1">
       <c r="B5" s="25" t="inlineStr">
@@ -1305,41 +1167,26 @@
       <c r="XFB5" s="23">
         <v>0.2</v>
       </c>
-      <c r="XFC5" s="23">
-        <v>0.3</v>
-      </c>
     </row>
     <row r="6">
       <c r="XFB6" s="23">
         <v>0.25</v>
       </c>
-      <c r="XFC6" s="23">
-        <v>0.35</v>
-      </c>
     </row>
     <row r="7">
       <c r="XFB7" s="23">
         <v>0.3</v>
       </c>
-      <c r="XFC7" s="23">
-        <v>0.4</v>
-      </c>
     </row>
     <row r="8">
       <c r="XFB8" s="23">
         <v>0.35</v>
       </c>
-      <c r="XFC8" s="23">
-        <v>0.45</v>
-      </c>
     </row>
     <row r="9">
       <c r="XFB9" s="23">
         <v>0.4</v>
       </c>
-      <c r="XFC9" s="23">
-        <v>0.5</v>
-      </c>
     </row>
     <row r="10" ht="27.8" customHeight="1">
       <c r="B10" s="26" t="inlineStr">
@@ -1375,9 +1222,6 @@
       <c r="XFB10" s="23">
         <v>0.45</v>
       </c>
-      <c r="XFC10" s="23">
-        <v>0.55</v>
-      </c>
     </row>
     <row r="11" ht="27.8" customHeight="1">
       <c r="B11" s="27" t="inlineStr">
@@ -1391,7 +1235,7 @@
         </is>
       </c>
       <c r="D11" s="29">
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
       <c r="F11" s="27" t="inlineStr">
         <is>
@@ -1409,9 +1253,6 @@
       <c r="XFB11" s="23">
         <v>0.5</v>
       </c>
-      <c r="XFC11" s="23">
-        <v>0.6</v>
-      </c>
     </row>
     <row r="12" ht="27.8" customHeight="1">
       <c r="B12" s="27" t="inlineStr">
@@ -1425,7 +1266,7 @@
         </is>
       </c>
       <c r="D12" s="29">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="F12" s="24" t="inlineStr">
         <is>
@@ -1437,9 +1278,6 @@
       <c r="XFB12" s="23">
         <v>0.55</v>
       </c>
-      <c r="XFC12" s="23">
-        <v>0.65</v>
-      </c>
     </row>
     <row r="13" ht="29.2" customHeight="1">
       <c r="B13" s="30" t="inlineStr">
@@ -1454,19 +1292,20 @@
       <c r="XFB13" s="23">
         <v>0.6</v>
       </c>
-      <c r="XFC13" s="23">
-        <v>0.7</v>
-      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="B14" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAMPAIGN BUDGET</t>
-        </is>
-      </c>
-      <c r="C14" s="30"/>
+          <t xml:space="preserve">BUDGET</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Your marketing for the year (at most €1,022,000)</t>
+        </is>
+      </c>
       <c r="D14" s="32">
-        <f>D23*D24</f>
+        <v>613000</v>
       </c>
       <c r="F14" s="34" t="inlineStr">
         <is>
@@ -1477,12 +1316,10 @@
       <c r="H14" s="34"/>
       <c r="I14" s="34"/>
       <c r="J14" s="34"/>
+      <c r="K14" s="34"/>
       <c r="XFB14" s="23">
         <v>0.65</v>
       </c>
-      <c r="XFC14" s="23">
-        <v>0.75</v>
-      </c>
     </row>
     <row r="15">
       <c r="F15" s="34" t="inlineStr">
@@ -1510,14 +1347,24 @@
           <t xml:space="preserve">Hit Ratio</t>
         </is>
       </c>
+      <c r="K15" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Weight</t>
+        </is>
+      </c>
       <c r="XFB15" s="23">
         <v>0.7</v>
       </c>
-      <c r="XFC15" s="23">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="16">
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customers per gift = reach × weight × interest × click × hit ratio.
+Each gift can serve at most (offer budget × its weight) ÷ its cost customers.</t>
+        </is>
+      </c>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
       <c r="F16" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">Discount on concert/event</t>
@@ -1535,14 +1382,17 @@
       <c r="J16" s="36">
         <v>0.1</v>
       </c>
+      <c r="K16" s="29">
+        <v>0.2</v>
+      </c>
       <c r="XFB16" s="23">
         <v>0.75</v>
       </c>
-      <c r="XFC16" s="23">
-        <v>0.85</v>
-      </c>
-    </row>
-    <row r="17">
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
       <c r="F17" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">Restaurant gift card</t>
@@ -1560,14 +1410,14 @@
       <c r="J17" s="36">
         <v>0.07</v>
       </c>
+      <c r="K17" s="29">
+        <v>0.4</v>
+      </c>
       <c r="XFB17" s="23">
         <v>0.8</v>
       </c>
-      <c r="XFC17" s="23">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="18">
+    </row>
+    <row r="18" ht="24" customHeight="1">
       <c r="F18" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">Coffee gift card</t>
@@ -1585,12 +1435,12 @@
       <c r="J18" s="36">
         <v>0.09</v>
       </c>
+      <c r="K18" s="29">
+        <v>0.3</v>
+      </c>
       <c r="XFB18" s="23">
         <v>0.85</v>
       </c>
-      <c r="XFC18" s="23">
-        <v>0.95</v>
-      </c>
     </row>
     <row r="19" ht="14.4" customHeight="1">
       <c r="F19" s="35" t="inlineStr">
@@ -1610,11 +1460,11 @@
       <c r="J19" s="36">
         <v>0.15</v>
       </c>
+      <c r="K19" s="29">
+        <v>0.1</v>
+      </c>
       <c r="XFB19" s="23">
         <v>0.9</v>
-      </c>
-      <c r="XFC19" s="23">
-        <v>1</v>
       </c>
     </row>
     <row r="20" ht="27.6" customHeight="1">
@@ -1627,6 +1477,9 @@
       <c r="H20" s="24"/>
       <c r="I20" s="24"/>
       <c r="J20" s="24"/>
+      <c r="K20" s="31">
+        <f>SUM(K16:K19)</f>
+      </c>
       <c r="XFB20" s="23">
         <v>0.95</v>
       </c>
@@ -1636,396 +1489,40 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" ht="27.8" customHeight="1">
-      <c r="B22" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Marketing</t>
-        </is>
-      </c>
-      <c r="C22" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Description</t>
-        </is>
-      </c>
-      <c r="D22" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value</t>
-        </is>
-      </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SELECTED OFFER</t>
-        </is>
-      </c>
-      <c r="G22" s="38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Restaurant gift card</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="24.8" customHeight="1">
-      <c r="B23" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Budget</t>
-        </is>
-      </c>
-      <c r="C23" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total marketing for the year, from the decision budget</t>
-        </is>
-      </c>
-      <c r="D23" s="39">
-        <v>460000</v>
-      </c>
-    </row>
-    <row r="24" ht="24.8" customHeight="1">
-      <c r="B24" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Campaign share</t>
-        </is>
-      </c>
-      <c r="C24" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Runs the digital campaign; the rest buys channel visibility</t>
-        </is>
-      </c>
-      <c r="D24" s="29">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="26" ht="27.8" customHeight="1">
-      <c r="B26" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Channel</t>
-        </is>
-      </c>
-      <c r="C26" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Description</t>
-        </is>
-      </c>
-      <c r="D26" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Share</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="21.8" customHeight="1">
-      <c r="B27" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Agency</t>
-        </is>
-      </c>
-      <c r="C27" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Agent marketing support</t>
-        </is>
-      </c>
-      <c r="D27" s="29">
-        <v>0.45</v>
-      </c>
-    </row>
-    <row r="28" ht="21.8" customHeight="1">
-      <c r="B28" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bank</t>
-        </is>
-      </c>
-      <c r="C28" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bancassurance visibility</t>
-        </is>
-      </c>
-      <c r="D28" s="29">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="29" ht="21.8" customHeight="1">
-      <c r="B29" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Digital</t>
-        </is>
-      </c>
-      <c r="C29" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Online visibility (outside the campaign)</t>
-        </is>
-      </c>
-      <c r="D29" s="29">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="30" ht="21.8" customHeight="1">
-      <c r="B30" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Broker</t>
-        </is>
-      </c>
-      <c r="C30" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Broker support</t>
-        </is>
-      </c>
-      <c r="D30" s="29">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="31" ht="27.8" customHeight="1">
-      <c r="B31" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TOTAL</t>
-        </is>
-      </c>
-      <c r="C31" s="30"/>
-      <c r="D31" s="31">
-        <f>SUM(D27:D30)</f>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="8">
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B3:H3"/>
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B16:D17"/>
     <mergeCell ref="F12:H12"/>
-    <mergeCell ref="F14:J14"/>
+    <mergeCell ref="F14:K14"/>
     <mergeCell ref="F20:J20"/>
-    <mergeCell ref="B31:C31"/>
   </mergeCells>
   <conditionalFormatting sqref="D13">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="notEqual">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D31">
+  <conditionalFormatting sqref="K20">
     <cfRule type="cellIs" dxfId="0" priority="2" operator="notEqual">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Pick a share from the list (steps of 5%)." sqref="D11:D12 D24">
+  <conditionalFormatting sqref="D14">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
+      <formula>1022000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Pick a share from the list (steps of 5%)." sqref="D11:D12 K16:K19">
       <formula1>PercentageList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Pick a share from the list (at least 10%)." sqref="D27:D30">
-      <formula1>FocusList</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Pick one of the offers." sqref="G22">
-      <formula1>OfferList</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" error="Enter 0 to 1022000." sqref="D23">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" error="Enter 0 to 1022000." sqref="D14">
       <formula1>0</formula1>
       <formula2>1022000</formula2>
     </dataValidation>
   </dataValidations>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr>
-    <tabColor rgb="FF004894"/>
-  </sheetPr>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="3.9" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="45.4" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="11" max="11" width="4.9" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="XFD1" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="35.2" customHeight="1">
-      <c r="B2" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CLAIM - BUDGET ALLOCATION</t>
-        </is>
-      </c>
-      <c r="XFD2" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="24.8" customHeight="1">
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Define the claims operations budget and the reinsurance treaty</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="27.8" customHeight="1">
-      <c r="B5" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">📊 CLAIMS OPERATIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="26.2" customHeight="1">
-      <c r="B7" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PARAMETER</t>
-        </is>
-      </c>
-      <c r="C7" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DESCRIPTION</t>
-        </is>
-      </c>
-      <c r="D7" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VALUE</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="26.2" customHeight="1">
-      <c r="B8" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Claims Operations</t>
-        </is>
-      </c>
-      <c r="C8" s="45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Claims-handling capacity. Too little hurts satisfaction (NPS) and leaks claims cost.</t>
-        </is>
-      </c>
-      <c r="D8" s="46">
-        <v>429000</v>
-      </c>
-    </row>
-    <row r="9" ht="26.2" customHeight="1">
-      <c r="B9" s="47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Marketing Budget</t>
-        </is>
-      </c>
-      <c r="C9" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From the Marketing sheet</t>
-        </is>
-      </c>
-      <c r="D9" s="49">
-        <f>Marketing!D23</f>
-      </c>
-    </row>
-    <row r="10" ht="26.2" customHeight="1">
-      <c r="B10" s="47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinsurance Fee</t>
-        </is>
-      </c>
-      <c r="C10" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Paid from the budget if the treaty is chosen</t>
-        </is>
-      </c>
-      <c r="D10" s="49">
-        <f>IF(D17="Yes",128000,0)</f>
-      </c>
-    </row>
-    <row r="11" ht="26.2" customHeight="1">
-      <c r="B11" s="47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Decision Budget</t>
-        </is>
-      </c>
-      <c r="C11" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The most you can spend in the year</t>
-        </is>
-      </c>
-      <c r="D11" s="49">
-        <v>1022000</v>
-      </c>
-    </row>
-    <row r="12" ht="27.8" customHeight="1">
-      <c r="B12" s="50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TOTAL USED</t>
-        </is>
-      </c>
-      <c r="C12" s="51"/>
-      <c r="D12" s="52">
-        <f>D8+D9+D10</f>
-      </c>
-    </row>
-    <row r="14" ht="27.8" customHeight="1">
-      <c r="B14" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">🔄 REINSURANCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="26.2" customHeight="1">
-      <c r="B16" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PARAMETER</t>
-        </is>
-      </c>
-      <c r="C16" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DESCRIPTION</t>
-        </is>
-      </c>
-      <c r="D16" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VALUE</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="27.8" customHeight="1">
-      <c r="B17" s="53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quota-share Reinsurance</t>
-        </is>
-      </c>
-      <c r="C17" s="54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cedes 30% of premium and claims for a 25% commission; costs €128,000</t>
-        </is>
-      </c>
-      <c r="D17" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">💡 Note: All choices are selected from dropdowns. The total used must not exceed the decision budget; the reinsurance holds for the whole year.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="B19:I19"/>
-  </mergeCells>
-  <conditionalFormatting sqref="D12">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
-      <formula>D11</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" error="Enter 0 to 1022000." sqref="D8">
-      <formula1>0</formula1>
-      <formula2>1022000</formula2>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Choose Yes or No." sqref="D17">
-      <formula1>YesNoList</formula1>
-    </dataValidation>
-  </dataValidations>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Marketing cap of €500k per team
At the default market size every team can spend at most €500k on the
campaign (it still scales with the policy count). The old €1.02m let a
full campaign bring half of a team's book; now it is about a quarter.
Samples rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/samples/casco-decision-sample.xlsx
+++ b/dist/samples/casco-decision-sample.xlsx
@@ -554,7 +554,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">The marketing budget must stay within €1,022,000.</t>
+          <t xml:space="preserve">The marketing budget must stay within €500,000.</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1143,7 @@
     <row r="3" ht="37.2" customHeight="1">
       <c r="B3" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">You have a budget of up to €1,022,000. You will split this among media &amp; offer.
+          <t xml:space="preserve">You have a budget of up to €500,000. You will split this among media &amp; offer.
 Sum should equal to 100%. Then weight the gifts: their sum should also equal to 100%.</t>
         </is>
       </c>
@@ -1301,11 +1301,11 @@
       </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Your marketing for the year (at most €1,022,000)</t>
+          <t xml:space="preserve">Your marketing for the year (at most €500,000)</t>
         </is>
       </c>
       <c r="D14" s="32">
-        <v>613000</v>
+        <v>300000</v>
       </c>
       <c r="F14" s="34" t="inlineStr">
         <is>
@@ -1512,16 +1512,16 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="D14">
     <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
-      <formula>1022000</formula>
+      <formula>500000</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Pick a share from the list (steps of 5%)." sqref="D11:D12 K16:K19">
       <formula1>PercentageList</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" error="Enter 0 to 1022000." sqref="D14">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" error="Enter 0 to 500000." sqref="D14">
       <formula1>0</formula1>
-      <formula2>1022000</formula2>
+      <formula2>500000</formula2>
     </dataValidation>
   </dataValidations>
 </worksheet>

</xml_diff>

<commit_message>
A simpler team screen; shares are any percentage
The team device now shows one thing at a time: a title, one line and at most two buttons, with optional links below; the roadmap, step boxes and plan summary are gone. Media share and gift weights no longer need steps of 5: any percentage from 0 to 100 is valid and the weights still total 100. The decision file takes typed percentages instead of a dropdown, and the samples are rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/samples/casco-decision-sample.xlsx
+++ b/dist/samples/casco-decision-sample.xlsx
@@ -11,7 +11,6 @@
   </sheets>
   <definedNames>
     <definedName name="CoefficientList">Premium!$XFD$1:$XFD$41</definedName>
-    <definedName name="PercentageList">Marketing!$XFB$1:$XFB$21</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -530,7 +529,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coefficients, shares and choices are selected from dropdown lists.</t>
+          <t xml:space="preserve">Coefficients are picked from dropdown lists; shares are typed in as percentages (any value from 0% to 100%).</t>
         </is>
       </c>
     </row>
@@ -1126,20 +1125,12 @@
     <col min="12" max="12" width="11.3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="XFB1" s="23">
-        <v>0</v>
-      </c>
-    </row>
     <row r="2" ht="35.2" customHeight="1">
       <c r="B2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">MARKETING - MEDIA &amp; OFFER</t>
         </is>
       </c>
-      <c r="XFB2" s="23">
-        <v>0.05</v>
-      </c>
     </row>
     <row r="3" ht="37.2" customHeight="1">
       <c r="B3" s="24" t="inlineStr">
@@ -1147,14 +1138,6 @@
           <t xml:space="preserve">You have two budgets of up to €250,000 each: January–June and July–December. Nothing carries over from one to the other.
 Split marketing among media &amp; offer (sum = 100%). Then weight the gifts: their sum should also equal 100%.</t>
         </is>
-      </c>
-      <c r="XFB3" s="23">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="XFB4" s="23">
-        <v>0.15</v>
       </c>
     </row>
     <row r="5" ht="42.6" customHeight="1">
@@ -1165,29 +1148,6 @@
 Target Group: Joyful Disregarders (21% of 18-55 digital users)</t>
         </is>
       </c>
-      <c r="XFB5" s="23">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="XFB6" s="23">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="XFB7" s="23">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="XFB8" s="23">
-        <v>0.35</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="XFB9" s="23">
-        <v>0.4</v>
-      </c>
     </row>
     <row r="10" ht="27.8" customHeight="1">
       <c r="B10" s="26" t="inlineStr">
@@ -1220,9 +1180,6 @@
           <t xml:space="preserve">Cost</t>
         </is>
       </c>
-      <c r="XFB10" s="23">
-        <v>0.45</v>
-      </c>
     </row>
     <row r="11" ht="27.8" customHeight="1">
       <c r="B11" s="27" t="inlineStr">
@@ -1251,9 +1208,6 @@
       <c r="H11" s="33">
         <v>10</v>
       </c>
-      <c r="XFB11" s="23">
-        <v>0.5</v>
-      </c>
     </row>
     <row r="12" ht="27.8" customHeight="1">
       <c r="B12" s="27" t="inlineStr">
@@ -1276,9 +1230,6 @@
       </c>
       <c r="G12" s="24"/>
       <c r="H12" s="24"/>
-      <c r="XFB12" s="23">
-        <v>0.55</v>
-      </c>
     </row>
     <row r="13" ht="29.2" customHeight="1">
       <c r="B13" s="30" t="inlineStr">
@@ -1289,9 +1240,6 @@
       <c r="C13" s="30"/>
       <c r="D13" s="31">
         <f>D11+D12</f>
-      </c>
-      <c r="XFB13" s="23">
-        <v>0.6</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
@@ -1318,9 +1266,6 @@
       <c r="I14" s="34"/>
       <c r="J14" s="34"/>
       <c r="K14" s="34"/>
-      <c r="XFB14" s="23">
-        <v>0.65</v>
-      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="30"/>
@@ -1362,9 +1307,6 @@
           <t xml:space="preserve">Weight</t>
         </is>
       </c>
-      <c r="XFB15" s="23">
-        <v>0.7</v>
-      </c>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="B16" s="24" t="inlineStr">
@@ -1394,9 +1336,6 @@
       </c>
       <c r="K16" s="29">
         <v>0.2</v>
-      </c>
-      <c r="XFB16" s="23">
-        <v>0.75</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
@@ -1423,9 +1362,6 @@
       <c r="K17" s="29">
         <v>0.4</v>
       </c>
-      <c r="XFB17" s="23">
-        <v>0.8</v>
-      </c>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="F18" s="35" t="inlineStr">
@@ -1448,9 +1384,6 @@
       <c r="K18" s="29">
         <v>0.3</v>
       </c>
-      <c r="XFB18" s="23">
-        <v>0.85</v>
-      </c>
     </row>
     <row r="19" ht="14.4" customHeight="1">
       <c r="F19" s="35" t="inlineStr">
@@ -1472,9 +1405,6 @@
       </c>
       <c r="K19" s="29">
         <v>0.1</v>
-      </c>
-      <c r="XFB19" s="23">
-        <v>0.9</v>
       </c>
     </row>
     <row r="20" ht="27.6" customHeight="1">
@@ -1489,14 +1419,6 @@
       <c r="J20" s="24"/>
       <c r="K20" s="31">
         <f>SUM(K16:K19)</f>
-      </c>
-      <c r="XFB20" s="23">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="XFB21" s="23">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1527,8 +1449,9 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Pick a share from the list (steps of 5%)." sqref="D11:D12 K16:K19">
-      <formula1>PercentageList</formula1>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" error="Enter a percentage from 0% to 100%." sqref="D11:D12 K16:K19">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
     </dataValidation>
     <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" error="Enter 0 to 250000." sqref="D14">
       <formula1>0</formula1>

</xml_diff>

<commit_message>
One trophy by total points; bankruptcy above a 135% combined ratio
Profit points and premium points each give nothing below their floor, 50 at it and 100 at their target (profit €0 to €1M, gross premium €4M to €8M, pro-rated during the year); the score is their sum and one trophy goes by it, ties by profit. A combined ratio above 135% is bankruptcy: the team is ranked last and stamped on the results table and the final. The results page is the trophy table with the points. The decision file has one marketing cell per half-year; the half-year review file's cell sets July–December. The audit workbook follows and matches the app in Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/samples/casco-decision-sample.xlsx
+++ b/dist/samples/casco-decision-sample.xlsx
@@ -492,7 +492,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select segment-based coefficients (0.50 - 2.50 range, 0.05 increments)</t>
+          <t xml:space="preserve">Select segment-based coefficients (0,50 - 2,50 range, 0,05 increments)</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Set the two half-year marketing budgets, split them among media &amp; offer (total must = 100%) and weight the gifts (total must = 100%)</t>
+          <t xml:space="preserve">Set the marketing budget per half-year, split it among media &amp; offer (total must = 100%) and weight the gifts (total must = 100%)</t>
         </is>
       </c>
     </row>
@@ -553,7 +553,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marketing has two budgets of up to €250,000 each: January–June and July–December. Each is spent evenly over its six months; what is not spent stays in profit, nothing carries over.</t>
+          <t xml:space="preserve">The marketing budget is one amount per half-year, up to €250.000: it runs January–June and again July–December, unless you set a new amount at the half-year review. What is not spent stays in profit; nothing carries over.</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Costs: claims; 5% of premium for running the business; the channel commission on premium (Agency 5%, Bank 10%, Digital 2%, Broker 10%); a fixed €500,000 a year; and the marketing you actually spend.</t>
+          <t xml:space="preserve">Costs: claims; 5% of premium for running the business; the channel commission on premium (Agency 5%, Bank 10%, Digital 2%, Broker 10%); a fixed €500.000 a year; and the marketing you actually spend.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
     <row r="3" ht="24.8" customHeight="1">
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select coefficient between 0.50 - 2.50 for each segment</t>
+          <t xml:space="preserve">Select coefficient between 0,50 - 2,50 for each segment</t>
         </is>
       </c>
       <c r="XFD3" s="23">
@@ -1135,7 +1135,7 @@
     <row r="3" ht="37.2" customHeight="1">
       <c r="B3" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">You have two budgets of up to €250,000 each: January–June and July–December. Nothing carries over from one to the other.
+          <t xml:space="preserve">Enter one budget per half-year, up to €250.000. It runs January–June and again July–December unless you change it at the half-year review.
 Split marketing among media &amp; offer (sum = 100%). Then weight the gifts: their sum should also equal 100%.</t>
         </is>
       </c>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">January–June (at most €250,000)</t>
+          <t xml:space="preserve">Budget per half-year (at most €250.000)</t>
         </is>
       </c>
       <c r="D14" s="32">
@@ -1267,16 +1267,7 @@
       <c r="J14" s="34"/>
       <c r="K14" s="34"/>
     </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="B15" s="30"/>
-      <c r="C15" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">July–December (at most €250,000)</t>
-        </is>
-      </c>
-      <c r="D15" s="32">
-        <v>150000</v>
-      </c>
+    <row r="15">
       <c r="F15" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">Possible Offers</t>
@@ -1422,12 +1413,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="7">
     <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B3:H3"/>
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:B15"/>
     <mergeCell ref="B16:D17"/>
     <mergeCell ref="F12:H12"/>
     <mergeCell ref="F14:K14"/>
@@ -1443,12 +1432,12 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D14:D15">
+  <conditionalFormatting sqref="D14">
     <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
       <formula>250000</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
+  <dataValidations count="2">
     <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" error="Enter a percentage from 0% to 100%." sqref="D11:D12 K16:K19">
       <formula1>0</formula1>
       <formula2>1</formula2>
@@ -1457,10 +1446,6 @@
       <formula1>0</formula1>
       <formula2>250000</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showErrorMessage="1" error="Enter 0 to 250000." sqref="D15">
-      <formula1>0</formula1>
-      <formula2>250000</formula2>
-    </dataValidation>
   </dataValidations>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Market share scoring, clean templates, private plans on stage
The second score component is market share among the teams: no points below 15%, 50 at 15%, 100 at 20%, not pro-rated; profit points are unchanged. A fresh template is clean: amounts and shares are empty, coefficients 1.00, and every input cell is yellow; a handed-in plan or the half-year review copy still comes back filled. The stage no longer shows teams' plans, only that a strategy was received. The stage lanes show the combined ratio and the policy count instead of points and campaign customers, while the order stays the trophy's. The communication asset is no longer labelled optional.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/samples/casco-decision-sample.xlsx
+++ b/dist/samples/casco-decision-sample.xlsx
@@ -340,7 +340,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -355,10 +355,10 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -370,19 +370,19 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -565,7 +565,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Costs: claims; 5% of premium for running the business; the channel commission on premium (Agency 5%, Bank 10%, Digital 2%, Broker 10%); a fixed €500.000 a year; and the marketing you actually spend.</t>
+          <t xml:space="preserve">Costs: claims; 5% of premium for running the business; the channel commission on premium (Agency 5%, Bank 10%, Digital 2%, Broker 10%); a fixed €200.000 a year; and the marketing you actually spend.</t>
         </is>
       </c>
     </row>

</xml_diff>